<commit_message>
docs: add 适用方向/Direction column (payables/receivables/both) to rule sheets; scope note on both architecture slides
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Payment Monitoring Scenarios-0709.xlsx
+++ b/docs/Payment Monitoring Scenarios-0709.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <name val="等线"/>
       <charset val="134"/>
@@ -211,6 +211,10 @@
       <family val="2"/>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="11">
@@ -438,7 +442,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="123">
+  <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -796,6 +800,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1160,7 +1170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M33"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.1640625" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="4" min="1" max="1"/>
@@ -1174,6 +1184,7 @@
     <col width="8.1640625" customWidth="1" style="4" min="10" max="10"/>
     <col width="28.6640625" customWidth="1" style="4" min="11" max="11"/>
     <col width="8.1640625" customWidth="1" style="4" min="12" max="16384"/>
+    <col width="22" customWidth="1" style="69" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="69">
@@ -1242,6 +1253,11 @@
           <t>Data from</t>
         </is>
       </c>
+      <c r="N1" s="123" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
     </row>
     <row r="2" hidden="1" ht="80" customHeight="1" s="69">
       <c r="A2" s="9" t="inlineStr">
@@ -1300,6 +1316,11 @@
           <t>External Database</t>
         </is>
       </c>
+      <c r="N2" s="124" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
     </row>
     <row r="3" hidden="1" ht="48" customHeight="1" s="69">
       <c r="A3" s="9" t="inlineStr">
@@ -1354,6 +1375,11 @@
           <t>External Database</t>
         </is>
       </c>
+      <c r="N3" s="124" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
     </row>
     <row r="4" hidden="1" ht="48" customHeight="1" s="69">
       <c r="A4" s="9" t="inlineStr">
@@ -1413,6 +1439,11 @@
           <t>tax havens list</t>
         </is>
       </c>
+      <c r="N4" s="124" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
     </row>
     <row r="5" hidden="1" ht="64" customHeight="1" s="69">
       <c r="A5" s="9" t="inlineStr">
@@ -1467,6 +1498,11 @@
           <t>AI Screening Tool</t>
         </is>
       </c>
+      <c r="N5" s="124" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
     </row>
     <row r="6" hidden="1" ht="102" customHeight="1" s="69">
       <c r="A6" s="9" t="inlineStr">
@@ -1521,6 +1557,11 @@
           <t>AI Screening Tool</t>
         </is>
       </c>
+      <c r="N6" s="124" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
     </row>
     <row r="7" hidden="1" ht="96" customHeight="1" s="69">
       <c r="A7" s="9" t="inlineStr">
@@ -1577,6 +1618,11 @@
           <t>External Database</t>
         </is>
       </c>
+      <c r="N7" s="124" t="inlineStr">
+        <is>
+          <t>Both — currently payables only</t>
+        </is>
+      </c>
     </row>
     <row r="8" hidden="1" ht="96" customHeight="1" s="69">
       <c r="A8" s="13" t="inlineStr">
@@ -1638,6 +1684,11 @@
           <t>company code; ship from;Remit To Address; contract region</t>
         </is>
       </c>
+      <c r="N8" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="29.25" customHeight="1" s="69">
       <c r="A9" s="13" t="inlineStr">
@@ -1685,6 +1736,11 @@
       <c r="K9" s="4" t="inlineStr">
         <is>
           <t>Coding: only happens in LGAP, normal scenario</t>
+        </is>
+      </c>
+      <c r="N9" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
         </is>
       </c>
     </row>
@@ -1739,6 +1795,11 @@
           <t>ML</t>
         </is>
       </c>
+      <c r="N10" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="11" hidden="1" ht="80" customHeight="1" s="69">
       <c r="A11" s="9" t="inlineStr">
@@ -1791,6 +1852,11 @@
       <c r="K11" s="4" t="inlineStr">
         <is>
           <t>ML</t>
+        </is>
+      </c>
+      <c r="N11" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
         </is>
       </c>
     </row>
@@ -1846,6 +1912,11 @@
           <t>ML</t>
         </is>
       </c>
+      <c r="N12" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="96" customHeight="1" s="69">
       <c r="A13" s="13" t="inlineStr">
@@ -1902,6 +1973,11 @@
           <t>Payer's weekends or holidays.</t>
         </is>
       </c>
+      <c r="N13" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="112" customHeight="1" s="69">
       <c r="A14" s="9" t="inlineStr">
@@ -1949,6 +2025,11 @@
         </is>
       </c>
       <c r="J14" s="11" t="n"/>
+      <c r="N14" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="15" hidden="1" ht="30.75" customFormat="1" customHeight="1" s="25">
       <c r="A15" s="26" t="inlineStr">
@@ -1995,6 +2076,11 @@
         </is>
       </c>
       <c r="J15" s="24" t="n"/>
+      <c r="N15" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="112" customFormat="1" customHeight="1" s="20">
       <c r="A16" s="21" t="inlineStr">
@@ -2051,6 +2137,11 @@
           <t>ML:Trend monitor</t>
         </is>
       </c>
+      <c r="N16" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="48" customFormat="1" customHeight="1" s="20">
       <c r="A17" s="21" t="inlineStr">
@@ -2105,6 +2196,11 @@
           <t>ML:Trend monitor</t>
         </is>
       </c>
+      <c r="N17" s="124" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="64" customFormat="1" customHeight="1" s="20">
       <c r="A18" s="16" t="inlineStr">
@@ -2155,6 +2251,11 @@
           <t>？</t>
         </is>
       </c>
+      <c r="N18" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="19" hidden="1" ht="32" customFormat="1" customHeight="1" s="20">
       <c r="A19" s="16" t="inlineStr">
@@ -2205,6 +2306,11 @@
           <t>ML? maybe out of scope cuz Ariba will not maintain bank account. It's LGVM</t>
         </is>
       </c>
+      <c r="N19" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="20" hidden="1" ht="48" customFormat="1" customHeight="1" s="20">
       <c r="A20" s="16" t="inlineStr">
@@ -2255,6 +2361,11 @@
           <t>ML? maybe out of scope cuz Ariba will not maintain bank account. It's LGVM</t>
         </is>
       </c>
+      <c r="N20" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="32" customFormat="1" customHeight="1" s="20">
       <c r="A21" s="16" t="inlineStr">
@@ -2303,6 +2414,11 @@
       <c r="K21" s="20" t="inlineStr">
         <is>
           <t>Coding: only happens in LGAP</t>
+        </is>
+      </c>
+      <c r="N21" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
         </is>
       </c>
     </row>
@@ -2356,6 +2472,11 @@
           <t>ML:Trend monitor</t>
         </is>
       </c>
+      <c r="N22" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="32" customFormat="1" customHeight="1" s="20">
       <c r="A23" s="16" t="inlineStr">
@@ -2407,6 +2528,11 @@
           <t>ML:Trend monitor</t>
         </is>
       </c>
+      <c r="N23" s="124" t="inlineStr">
+        <is>
+          <t>Both — currently payables only</t>
+        </is>
+      </c>
     </row>
     <row r="24" hidden="1" ht="16" customFormat="1" customHeight="1" s="20">
       <c r="A24" s="16" t="inlineStr">
@@ -2456,6 +2582,11 @@
           <t>Inhouse Database</t>
         </is>
       </c>
+      <c r="N24" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="25" hidden="1" ht="102" customFormat="1" customHeight="1" s="20">
       <c r="A25" s="16" t="inlineStr">
@@ -2506,6 +2637,11 @@
           <t>AI Screening Tool</t>
         </is>
       </c>
+      <c r="N25" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="16" customFormat="1" customHeight="1" s="20">
       <c r="A26" s="16" t="inlineStr">
@@ -2555,6 +2691,11 @@
           <t>ML:Trend monitor</t>
         </is>
       </c>
+      <c r="N26" s="124" t="inlineStr">
+        <is>
+          <t>Receivables (customer) — out of current scope</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="16" customFormat="1" customHeight="1" s="20">
       <c r="A27" s="21" t="inlineStr">
@@ -2604,6 +2745,11 @@
           <t>External Database</t>
         </is>
       </c>
+      <c r="N27" s="124" t="inlineStr">
+        <is>
+          <t>Receivables (customer) — out of current scope</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="16" customFormat="1" customHeight="1" s="20">
       <c r="A28" s="21" t="inlineStr">
@@ -2657,6 +2803,11 @@
           <t>ML:Trend monitor</t>
         </is>
       </c>
+      <c r="N28" s="124" t="inlineStr">
+        <is>
+          <t>Receivables (cash banned on payables side)</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="17" customFormat="1" customHeight="1" s="20">
       <c r="A29" s="21" t="inlineStr">
@@ -2704,6 +2855,11 @@
       <c r="K29" s="20" t="inlineStr">
         <is>
           <t>threshold</t>
+        </is>
+      </c>
+      <c r="N29" s="124" t="inlineStr">
+        <is>
+          <t>Both (text reads receivables; DT treats as AP control)</t>
         </is>
       </c>
     </row>
@@ -4648,7 +4804,7 @@
     <col width="39.6640625" customWidth="1" style="69" min="13" max="13"/>
     <col width="41.6640625" customWidth="1" style="69" min="14" max="14"/>
     <col width="26.83203125" customWidth="1" style="69" min="16" max="16"/>
-    <col width="8.83203125" customWidth="1" style="69" min="17" max="17"/>
+    <col width="22" customWidth="1" style="69" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="69">
@@ -4732,6 +4888,11 @@
           <t>Questions</t>
         </is>
       </c>
+      <c r="Q1" s="74" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="96" customHeight="1" s="69">
       <c r="B2" s="75" t="inlineStr">
@@ -4811,6 +4972,11 @@
 Sanctions list ( )</t>
         </is>
       </c>
+      <c r="Q2" s="124" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="72" customHeight="1" s="69">
       <c r="B3" s="75" t="inlineStr">
@@ -4888,7 +5054,11 @@
 Basel AML Index</t>
         </is>
       </c>
-      <c r="Q3" s="83" t="n"/>
+      <c r="Q3" s="124" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="64" customHeight="1" s="69">
       <c r="B4" s="75" t="inlineStr">
@@ -4959,6 +5129,11 @@
       <c r="O4" s="79" t="inlineStr">
         <is>
           <t>Offshore list (https://ec.europa.eu/eurostat/statistics-explained/index.php?title=Glossary:List_of_offshore_financial_centres)</t>
+        </is>
+      </c>
+      <c r="Q4" s="124" t="inlineStr">
+        <is>
+          <t>Both</t>
         </is>
       </c>
     </row>
@@ -5032,6 +5207,11 @@
       <c r="O5" s="84" t="inlineStr">
         <is>
           <t>Litigation lookup: Tianyancha for China, Dow Jones for ROW</t>
+        </is>
+      </c>
+      <c r="Q5" s="124" t="inlineStr">
+        <is>
+          <t>Both</t>
         </is>
       </c>
     </row>
@@ -5107,6 +5287,11 @@
           <t>Tianyancha for China, Dow Jones for ROW</t>
         </is>
       </c>
+      <c r="Q6" s="124" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="72" customHeight="1" s="69">
       <c r="A7" s="85" t="inlineStr">
@@ -5184,6 +5369,11 @@
           <t>Principal place of business: Tianyancha for China, Dow Jones for ROW</t>
         </is>
       </c>
+      <c r="Q7" s="124" t="inlineStr">
+        <is>
+          <t>Both — currently payables only</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="54" customHeight="1" s="69">
       <c r="A8" s="85" t="inlineStr">
@@ -5264,6 +5454,11 @@
       <c r="P8" s="87" t="inlineStr">
         <is>
           <t>What is the difference from #7?</t>
+        </is>
+      </c>
+      <c r="Q8" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
         </is>
       </c>
     </row>
@@ -5326,6 +5521,11 @@
         </is>
       </c>
       <c r="O9" s="89" t="n"/>
+      <c r="Q9" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="126" customHeight="1" s="69">
       <c r="B10" s="75" t="inlineStr">
@@ -5395,6 +5595,11 @@
           <t>Business scope, registered capital etc.: Tianyancha for China, Dow Jones for ROW</t>
         </is>
       </c>
+      <c r="Q10" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="72" customHeight="1" s="69">
       <c r="A11" s="85" t="inlineStr">
@@ -5467,6 +5672,11 @@
       <c r="O11" s="84" t="inlineStr">
         <is>
           <t>Business scope, registered capital etc.: Tianyancha for China, Dow Jones for ROW</t>
+        </is>
+      </c>
+      <c r="Q11" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
         </is>
       </c>
     </row>
@@ -5535,6 +5745,11 @@
         </is>
       </c>
       <c r="O12" s="89" t="n"/>
+      <c r="Q12" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="54" customHeight="1" s="69">
       <c r="B13" s="75" t="inlineStr">
@@ -5601,6 +5816,11 @@
           <t>Public-holiday lookup tools per country</t>
         </is>
       </c>
+      <c r="Q13" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="108" customHeight="1" s="69">
       <c r="B14" s="75" t="inlineStr">
@@ -5665,6 +5885,11 @@
           <t>Business scope, registered capital etc.: Tianyancha for China, Dow Jones for ROW</t>
         </is>
       </c>
+      <c r="Q14" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="54" customHeight="1" s="69">
       <c r="A15" s="85" t="inlineStr">
@@ -5728,6 +5953,11 @@
       <c r="P15" s="82" t="inlineStr">
         <is>
           <t>How to verify historical invoices?</t>
+        </is>
+      </c>
+      <c r="Q15" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
         </is>
       </c>
     </row>
@@ -5756,6 +5986,11 @@
           <t>What is the threshold?</t>
         </is>
       </c>
+      <c r="Q17" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="36" customHeight="1" s="69">
       <c r="A18" s="85" t="n"/>
@@ -5782,6 +6017,11 @@
 Sudden surge: 500% payment increase.</t>
         </is>
       </c>
+      <c r="Q18" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="56" customHeight="1" s="69">
       <c r="A19" s="85" t="n"/>
@@ -5802,6 +6042,11 @@
       </c>
       <c r="F19" s="85" t="n"/>
       <c r="G19" s="83" t="n"/>
+      <c r="Q19" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="42" customHeight="1" s="69">
       <c r="A20" s="85" t="n"/>
@@ -5822,6 +6067,11 @@
       </c>
       <c r="F20" s="85" t="n"/>
       <c r="G20" s="83" t="n"/>
+      <c r="Q20" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="42" customHeight="1" s="69">
       <c r="A21" s="85" t="n"/>
@@ -5842,11 +6092,12 @@
       </c>
       <c r="F21" s="85" t="n"/>
       <c r="G21" s="83" t="n"/>
-    </row>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
+      <c r="Q21" s="124" t="inlineStr">
+        <is>
+          <t>Payables (vendor)</t>
+        </is>
+      </c>
+    </row>
     <row r="26" ht="198" customHeight="1" s="69">
       <c r="A26" s="71" t="inlineStr">
         <is>
@@ -5997,11 +6248,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
     <row r="36">
       <c r="N36" s="116" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: sync Legal-confirmation columns (R/S) to both Updated-0709-EN tabs
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Payment Monitoring Scenarios-0709.xlsx
+++ b/docs/Payment Monitoring Scenarios-0709.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="27">
+  <fonts count="29">
     <font>
       <name val="等线"/>
       <charset val="134"/>
@@ -215,6 +215,15 @@
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9.5"/>
     </font>
   </fonts>
   <fills count="11">
@@ -442,7 +451,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="125">
+  <cellXfs count="127">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -808,6 +817,10 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -4786,7 +4799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q39"/>
+  <dimension ref="A1:S39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.1640625" customWidth="1" style="69" min="1" max="1"/>
@@ -4805,6 +4818,8 @@
     <col width="41.6640625" customWidth="1" style="69" min="14" max="14"/>
     <col width="26.83203125" customWidth="1" style="69" min="16" max="16"/>
     <col width="22" customWidth="1" style="69" min="17" max="17"/>
+    <col width="52" customWidth="1" style="69" min="18" max="18"/>
+    <col width="42" customWidth="1" style="69" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1" s="69">
@@ -4893,6 +4908,16 @@
           <t>Direction</t>
         </is>
       </c>
+      <c r="R1" s="74" t="inlineStr">
+        <is>
+          <t>Legal Confirmation · Proposed Basis</t>
+        </is>
+      </c>
+      <c r="S1" s="74" t="inlineStr">
+        <is>
+          <t>Legal Confirmation · To Decide</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="96" customHeight="1" s="69">
       <c r="B2" s="75" t="inlineStr">
@@ -4977,6 +5002,20 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="R2" s="125" t="inlineStr">
+        <is>
+          <t>To confirm: (1) which country fields (2) CPI threshold (3) list ownership
+Candidates: registration country (S4 BP) / place of business / invoice country (Ariba|LGAP) / bank country (SWIFT parse)
+Proposal: check all four; any hit triggers; CPI &lt;40 = high risk; list maintained yearly by Brenda</t>
+        </is>
+      </c>
+      <c r="S2" s="125" t="inlineStr">
+        <is>
+          <t>(1) All-four-countries approach OK, or only some?
+(2) CPI threshold?
+(3) List refresh cycle &amp; owner</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="72" customHeight="1" s="69">
       <c r="B3" s="75" t="inlineStr">
@@ -5059,6 +5098,18 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="R3" s="125" t="inlineStr">
+        <is>
+          <t>To confirm: (1) does the grey list trigger too (2) which sanctions regimes
+Proposal: black + grey both trigger (grey at lower priority); sanctions base = OFAC + EU + UN</t>
+        </is>
+      </c>
+      <c r="S3" s="125" t="inlineStr">
+        <is>
+          <t>(1) Treat grey list same as black?
+(2) Which 'economic sanctions laws' (open question in K3)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="64" customHeight="1" s="69">
       <c r="B4" s="75" t="inlineStr">
@@ -5134,6 +5185,20 @@
       <c r="Q4" s="124" t="inlineStr">
         <is>
           <t>Both</t>
+        </is>
+      </c>
+      <c r="R4" s="125" t="inlineStr">
+        <is>
+          <t>* MAJOR ambiguity: which route does 'routed through' mean
+Candidates: a. goods route (Ariba PO has only ship-from/to; full route needs logistics TMS - unavailable) b. funds route (receiving/intermediary bank country, S4/SWIFT - available)
+Proposal: start with the FUNDS route (closer to laundering substance); approximate goods route by PO endpoints; use the EU offshore financial centres list</t>
+        </is>
+      </c>
+      <c r="S4" s="125" t="inlineStr">
+        <is>
+          <t>(1) Funds route, goods route, or both?
+(2) Endpoints-only (no full route) acceptable?
+(3) Confirm the offshore list</t>
         </is>
       </c>
     </row>
@@ -5212,6 +5277,20 @@
       <c r="Q5" s="124" t="inlineStr">
         <is>
           <t>Both</t>
+        </is>
+      </c>
+      <c r="R5" s="125" t="inlineStr">
+        <is>
+          <t>To confirm: (1) proceeding types &amp; lookback (2) which parties (3) internal records
+Candidates: Tianyancha (CN) / DJ (ROW) litigation; internal corrupt-party payment history (S4 AP) - but no 'known corrupt party' list exists today
+Proposal: corruption/fraud/ML-related only, last 5 years; company + legal rep + controlling shareholder</t>
+        </is>
+      </c>
+      <c r="S5" s="125" t="inlineStr">
+        <is>
+          <t>(1) Proceeding types &amp; years?
+(2) Party scope?
+(3) Which team owns the internal 'known corrupt party' list?</t>
         </is>
       </c>
     </row>
@@ -5292,6 +5371,19 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="R6" s="125" t="inlineStr">
+        <is>
+          <t>To confirm: (1) ownership depth &amp; threshold (2) PEP source
+Candidates: Tianyancha equity (CN) / DJ (ROW); PEP db = DJ; role list per D6
+Proposal: 2 levels deep; &gt;=10% stake or any D6 role; high-risk-jurisdiction PEP weighted up at investigation</t>
+        </is>
+      </c>
+      <c r="S6" s="125" t="inlineStr">
+        <is>
+          <t>(1) Depth &amp; stake threshold?
+(2) Is DJ's PEP db enough for Chinese officials?</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="72" customHeight="1" s="69">
       <c r="A7" s="85" t="inlineStr">
@@ -5374,6 +5466,19 @@
           <t>Both — currently payables only</t>
         </is>
       </c>
+      <c r="R7" s="125" t="inlineStr">
+        <is>
+          <t>To confirm: 'principal place of business' = registration country or actual?
+Candidates: a. registration country (S4 BP, internal) b. actual place of business (TYC/DJ, external)
+Proposal: detection uses registration country (automatable); actual place verified at investigation; bank country parsed from receiving-account SWIFT prefix (S4)</t>
+        </is>
+      </c>
+      <c r="S7" s="125" t="inlineStr">
+        <is>
+          <t>(1) Registration country acceptable as the basis? Which wins on conflict?
+(2) Judge per account when a vendor has several receiving accounts?</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="54" customHeight="1" s="69">
       <c r="A8" s="85" t="inlineStr">
@@ -5459,6 +5564,20 @@
       <c r="Q8" s="124" t="inlineStr">
         <is>
           <t>Payables (vendor)</t>
+        </is>
+      </c>
+      <c r="R8" s="125" t="inlineStr">
+        <is>
+          <t>* 'Invoice origin' = which field on the invoice
+Candidates: a. issuer address country b. remit-to country c. tax-ID country (VAT prefix); payer country = Lenovo company-code country (S4)
+Proposal: issuer address country as primary, tax-ID country as cross-check; boundary vs row 7: R7 = bank vs vendor, R8 = payer entity vs invoice (answers P8)</t>
+        </is>
+      </c>
+      <c r="S8" s="125" t="inlineStr">
+        <is>
+          <t>(1) Origin = issuer address? What if tax-ID country differs?
+(2) Agree with the R7/R8 boundary?
+(3) LGAP attachment invoices need OCR - acceptable? Confidence bar?</t>
         </is>
       </c>
     </row>
@@ -5524,6 +5643,17 @@
       <c r="Q9" s="124" t="inlineStr">
         <is>
           <t>Payables (vendor)</t>
+        </is>
+      </c>
+      <c r="R9" s="125" t="inlineStr">
+        <is>
+          <t>DT noted 'LGAP only, normal scenario'
+Proposal: no standalone alert; use as a risk feature in scoring only (no PO = one less 3-way-match defence)</t>
+        </is>
+      </c>
+      <c r="S9" s="125" t="inlineStr">
+        <is>
+          <t>Confirm: record-only? Or should non-PO payments outside specific expense types still alert?</t>
         </is>
       </c>
     </row>
@@ -5600,6 +5730,20 @@
           <t>Payables (vendor)</t>
         </is>
       </c>
+      <c r="R10" s="125" t="inlineStr">
+        <is>
+          <t>To confirm: (1) multiple threshold (2) window (3) no registered-capital concept abroad
+Candidates: registered capital = TYC/DJ (missing in some countries); PO history = Ariba; payments = S4 AP
+Proposal: rolling 12-month payments &gt; registered capital x10 triggers; abroad use headcount/revenue band or skip</t>
+        </is>
+      </c>
+      <c r="S10" s="125" t="inlineStr">
+        <is>
+          <t>(1) Multiple threshold?
+(2) 12-month window OK?
+(3) Overseas fallback acceptable?</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="72" customHeight="1" s="69">
       <c r="A11" s="85" t="inlineStr">
@@ -5677,6 +5821,20 @@
       <c r="Q11" s="124" t="inlineStr">
         <is>
           <t>Payables (vendor)</t>
+        </is>
+      </c>
+      <c r="R11" s="125" t="inlineStr">
+        <is>
+          <t>To confirm: (1) 'irrelevant' criterion (2) category granularity (3) LLM judgment acceptable?
+Candidates: business scope = TYC/DJ; category = Ariba commodity code (UNSPSC tree)
+Proposal: LLM semantic-relevance scoring with written rationale; start at top-level categories (fewer false positives)</t>
+        </is>
+      </c>
+      <c r="S11" s="125" t="inlineStr">
+        <is>
+          <t>(1) Accept LLM judgment? Confidence bar?
+(2) Top-level or detailed categories?
+(3) How to treat trading companies (very broad scope)?</t>
         </is>
       </c>
     </row>
@@ -5750,6 +5908,20 @@
           <t>Payables (vendor)</t>
         </is>
       </c>
+      <c r="R12" s="125" t="inlineStr">
+        <is>
+          <t>To confirm: (1) baseline (2) per-payment or cumulative (3) first-order-large case
+Candidates: onboarding date = S4 BP / Ariba SLP; payment history = S4 (incl. LGAP channel)
+Proposal: new = onboarded &lt;12 months; baseline = prior 6-month monthly average; monthly total &gt; baseline x5 triggers; separate absolute threshold for large first orders</t>
+        </is>
+      </c>
+      <c r="S12" s="125" t="inlineStr">
+        <is>
+          <t>(1) Baseline OK?
+(2) Absolute threshold for large first orders?
+(3) 500% (DT's suggestion) - does Legal agree?</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="54" customHeight="1" s="69">
       <c r="B13" s="75" t="inlineStr">
@@ -5821,6 +5993,19 @@
           <t>Payables (vendor)</t>
         </is>
       </c>
+      <c r="R13" s="125" t="inlineStr">
+        <is>
+          <t>To confirm: (1) which date (2) whose calendar
+Candidates: a. payment execution date (S4 clearing) b. invoice date c. request date (LGAP/Ariba)
+Proposal: use payment execution date (actual money movement; request/invoice dates over-alert); calendar of the payer country (O13 already leans payer side)</t>
+        </is>
+      </c>
+      <c r="S13" s="125" t="inlineStr">
+        <is>
+          <t>(1) Confirm the date basis?
+(2) Payer = Lenovo paying entity's country - confirm?</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="108" customHeight="1" s="69">
       <c r="B14" s="75" t="inlineStr">
@@ -5890,6 +6075,19 @@
           <t>Payables (vendor)</t>
         </is>
       </c>
+      <c r="R14" s="125" t="inlineStr">
+        <is>
+          <t>To confirm: (1) definition of 'apparent connection' (2) keep or drop
+Candidates: registered account = S4 vendor master; actual receiving account = payment request/document; connection via TYC/DJ equity
+Proposal: connection = same entity or &gt;=50%-owned affiliate (K14's own suggestion); drop if DT confirms LGAP hard control</t>
+        </is>
+      </c>
+      <c r="S14" s="125" t="inlineStr">
+        <is>
+          <t>(1) 50% threshold OK? Does group treasury collection count as connected?
+(2) Decide after DT's finding</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="54" customHeight="1" s="69">
       <c r="A15" s="85" t="inlineStr">
@@ -5958,6 +6156,20 @@
       <c r="Q15" s="124" t="inlineStr">
         <is>
           <t>Payables (vendor)</t>
+        </is>
+      </c>
+      <c r="R15" s="125" t="inlineStr">
+        <is>
+          <t>To confirm: (1) 'fake' criteria (CN vs ROW) (2) historical invoice checks (3) image availability
+Candidates: CN = tax-bureau verification platform (hard evidence); ROW = duplicate numbers (S4 AP) + sequential numbers + template/field anomalies (soft); images = Ariba Network / LGAP attachments
+Proposal: CN via tax verification; ROW: 3 soft checks route to manual review</t>
+        </is>
+      </c>
+      <c r="S15" s="125" t="inlineStr">
+        <is>
+          <t>(1) Do ROW soft checks still count as T1?
+(2) How far back for historical invoices?
+(3) Failed verification = fraud verdict directly?</t>
         </is>
       </c>
     </row>
@@ -6095,6 +6307,26 @@
       <c r="Q21" s="124" t="inlineStr">
         <is>
           <t>Payables (vendor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="126" t="inlineStr">
+        <is>
+          <t>Cross-rule</t>
+        </is>
+      </c>
+      <c r="R23" s="125" t="inlineStr">
+        <is>
+          <t>Cross-rule conventions
+Proposal: amounts converted to USD (payment-date FX); country-field precedence bank &gt; invoice &gt; registration (for discussion); SLA in calendar days</t>
+        </is>
+      </c>
+      <c r="S23" s="125" t="inlineStr">
+        <is>
+          <t>(1) Currency conversion basis?
+(2) Country-field precedence?
+(3) T1's 24h: calendar or business days?</t>
         </is>
       </c>
     </row>

</xml_diff>